<commit_message>
update names of variables
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Data.xlsx
+++ b/01_data/01_input_data/02_processed/Data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Gurobi_Projects\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7B96914-A6BF-402F-A80D-F4BB2E238F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73A7C8EC-76DE-44F4-9186-FE81C8A55A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-5070" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Nodes" sheetId="1" r:id="rId1"/>
@@ -1124,7 +1124,7 @@
         <v>0</v>
       </c>
       <c r="E16">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="F16">
         <v>5</v>
@@ -1150,7 +1150,7 @@
         <v>0</v>
       </c>
       <c r="E17">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="F17">
         <v>8</v>
@@ -1176,7 +1176,7 @@
         <v>0</v>
       </c>
       <c r="E18">
-        <v>35</v>
+        <v>70</v>
       </c>
       <c r="F18">
         <v>6</v>
@@ -1202,7 +1202,7 @@
         <v>0</v>
       </c>
       <c r="E19">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F19">
         <v>10</v>
@@ -1228,7 +1228,7 @@
         <v>0</v>
       </c>
       <c r="E20">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="F20">
         <v>7</v>
@@ -1254,7 +1254,7 @@
         <v>0</v>
       </c>
       <c r="E21">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="F21">
         <v>3</v>
@@ -1280,7 +1280,7 @@
         <v>0</v>
       </c>
       <c r="E22">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="F22">
         <v>1</v>
@@ -1306,7 +1306,7 @@
         <v>0</v>
       </c>
       <c r="E23">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="F23">
         <v>2</v>
@@ -1332,7 +1332,7 @@
         <v>0</v>
       </c>
       <c r="E24">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="F24">
         <v>3</v>
@@ -1358,7 +1358,7 @@
         <v>0</v>
       </c>
       <c r="E25">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F25">
         <v>5</v>
@@ -1384,7 +1384,7 @@
         <v>0</v>
       </c>
       <c r="E26">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F26">
         <v>4</v>
@@ -1410,7 +1410,7 @@
         <v>0</v>
       </c>
       <c r="E27">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F27">
         <v>7</v>
@@ -1436,7 +1436,7 @@
         <v>0</v>
       </c>
       <c r="E28">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F28">
         <v>5</v>
@@ -1462,7 +1462,7 @@
         <v>0</v>
       </c>
       <c r="E29">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F29">
         <v>2</v>

</xml_diff>

<commit_message>
update of the change variable to be edge specific
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Data.xlsx
+++ b/01_data/01_input_data/02_processed/Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73A7C8EC-76DE-44F4-9186-FE81C8A55A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1ECE662-2725-4288-B62F-EFDC6088D15A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="30">
   <si>
     <t>Supply Nodes</t>
   </si>
@@ -128,6 +128,9 @@
   </si>
   <si>
     <t>Hydrogen</t>
+  </si>
+  <si>
+    <t>conversion_capacity_factor</t>
   </si>
 </sst>
 </file>
@@ -717,10 +720,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C781A78E-EFEC-4F2E-A496-3B44BD173FD3}">
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -745,8 +748,11 @@
       <c r="H1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -771,8 +777,11 @@
       <c r="H2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>27</v>
       </c>
@@ -797,8 +806,11 @@
       <c r="H3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -823,8 +835,11 @@
       <c r="H4">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -849,8 +864,11 @@
       <c r="H5">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -875,8 +893,11 @@
       <c r="H6">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>27</v>
       </c>
@@ -901,8 +922,11 @@
       <c r="H7">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>27</v>
       </c>
@@ -927,8 +951,11 @@
       <c r="H8">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>27</v>
       </c>
@@ -953,8 +980,11 @@
       <c r="H9">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -979,8 +1009,11 @@
       <c r="H10">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>27</v>
       </c>
@@ -1005,8 +1038,11 @@
       <c r="H11">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>27</v>
       </c>
@@ -1031,8 +1067,11 @@
       <c r="H12">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>27</v>
       </c>
@@ -1057,8 +1096,11 @@
       <c r="H13">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>27</v>
       </c>
@@ -1083,8 +1125,11 @@
       <c r="H14">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>27</v>
       </c>
@@ -1109,8 +1154,11 @@
       <c r="H15">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>28</v>
       </c>
@@ -1135,8 +1183,11 @@
       <c r="H16">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>28</v>
       </c>
@@ -1161,8 +1212,11 @@
       <c r="H17">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>28</v>
       </c>
@@ -1187,8 +1241,11 @@
       <c r="H18">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I18">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>28</v>
       </c>
@@ -1213,8 +1270,11 @@
       <c r="H19">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>28</v>
       </c>
@@ -1239,8 +1299,11 @@
       <c r="H20">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>28</v>
       </c>
@@ -1265,8 +1328,11 @@
       <c r="H21">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I21">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>28</v>
       </c>
@@ -1291,8 +1357,11 @@
       <c r="H22">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>28</v>
       </c>
@@ -1317,8 +1386,11 @@
       <c r="H23">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I23">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>28</v>
       </c>
@@ -1343,8 +1415,11 @@
       <c r="H24">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I24">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>28</v>
       </c>
@@ -1369,8 +1444,11 @@
       <c r="H25">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>28</v>
       </c>
@@ -1395,8 +1473,11 @@
       <c r="H26">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I26">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>28</v>
       </c>
@@ -1421,8 +1502,11 @@
       <c r="H27">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I27">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>28</v>
       </c>
@@ -1447,8 +1531,11 @@
       <c r="H28">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I28">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>28</v>
       </c>
@@ -1472,6 +1559,9 @@
       </c>
       <c r="H29">
         <v>0.5</v>
+      </c>
+      <c r="I29">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>